<commit_message>
HVAC: credit solar gain in heat mode (author decision); recompute bounds and GT
Pending source review: the 20 Btu/h per ft2 glass value is still an unsourced
assumption. New HVAC bounds: cost $0.19-$3.21, environmental 0.97-17.59 lbs CO2.
Ground truth, HVAC RAG scores, fixed-default baseline, README, provenance and
tests updated. 12/105 winners and 16/105 rankings change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JVf7wf3sHYXwFDWcVM4QWD
</commit_message>
<xml_diff>
--- a/Output Files/Baselines/baseline_fixeddefault.xlsx
+++ b/Output Files/Baselines/baseline_fixeddefault.xlsx
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.71</v>
       </c>
       <c r="H2" t="n">
         <v>0.7</v>
@@ -570,7 +570,7 @@
         <v>0.77</v>
       </c>
       <c r="J2" t="n">
-        <v>0.785</v>
+        <v>0.714</v>
       </c>
       <c r="K2" t="n">
         <v>3</v>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="G3" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
@@ -633,7 +633,7 @@
         <v>0.84</v>
       </c>
       <c r="J3" t="n">
-        <v>0.872</v>
+        <v>0.8005</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.87</v>
+        <v>0.75</v>
       </c>
       <c r="G4" t="n">
-        <v>0.87</v>
+        <v>0.76</v>
       </c>
       <c r="H4" t="n">
         <v>0.7</v>
@@ -696,7 +696,7 @@
         <v>0.84</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8315</v>
+        <v>0.757</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="G5" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="H5" t="n">
         <v>0.78</v>
@@ -759,7 +759,7 @@
         <v>0.65</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8155</v>
+        <v>0.884</v>
       </c>
       <c r="K5" t="n">
         <v>2</v>
@@ -810,10 +810,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.83</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>0.83</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
@@ -822,7 +822,7 @@
         <v>0.65</v>
       </c>
       <c r="J6" t="n">
-        <v>0.837</v>
+        <v>0.9085</v>
       </c>
       <c r="K6" t="n">
         <v>1</v>
@@ -873,10 +873,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
       <c r="H7" t="n">
         <v>0.78</v>
@@ -885,7 +885,7 @@
         <v>0.65</v>
       </c>
       <c r="J7" t="n">
-        <v>0.7735</v>
+        <v>0.848</v>
       </c>
       <c r="K7" t="n">
         <v>3</v>
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="G8" t="n">
-        <v>0.68</v>
+        <v>0.59</v>
       </c>
       <c r="H8" t="n">
         <v>0.93</v>
@@ -948,7 +948,7 @@
         <v>0.84</v>
       </c>
       <c r="J8" t="n">
-        <v>0.751</v>
+        <v>0.6925</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
@@ -999,10 +999,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.71</v>
+        <v>0.61</v>
       </c>
       <c r="G9" t="n">
-        <v>0.71</v>
+        <v>0.62</v>
       </c>
       <c r="H9" t="n">
         <v>0.7</v>
@@ -1011,7 +1011,7 @@
         <v>0.84</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7275</v>
+        <v>0.666</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -1062,10 +1062,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="G10" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="H10" t="n">
         <v>0.41</v>
@@ -1074,7 +1074,7 @@
         <v>0.77</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.617</v>
       </c>
       <c r="K10" t="n">
         <v>3</v>
@@ -1125,10 +1125,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.67</v>
+        <v>0.89</v>
       </c>
       <c r="G11" t="n">
-        <v>0.67</v>
+        <v>0.89</v>
       </c>
       <c r="H11" t="n">
         <v>0.51</v>
@@ -1137,7 +1137,7 @@
         <v>0.65</v>
       </c>
       <c r="J11" t="n">
-        <v>0.635</v>
+        <v>0.778</v>
       </c>
       <c r="K11" t="n">
         <v>3</v>
@@ -1188,10 +1188,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.61</v>
+        <v>0.84</v>
       </c>
       <c r="G12" t="n">
-        <v>0.62</v>
+        <v>0.84</v>
       </c>
       <c r="H12" t="n">
         <v>0.78</v>
@@ -1200,7 +1200,7 @@
         <v>0.65</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6535</v>
+        <v>0.7995</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="G13" t="n">
-        <v>0.57</v>
+        <v>0.79</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -1263,7 +1263,7 @@
         <v>0.65</v>
       </c>
       <c r="J13" t="n">
-        <v>0.665</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
@@ -1314,10 +1314,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="G14" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="H14" t="n">
         <v>0.86</v>
@@ -1326,7 +1326,7 @@
         <v>0.84</v>
       </c>
       <c r="J14" t="n">
-        <v>0.8115</v>
+        <v>0.74</v>
       </c>
       <c r="K14" t="n">
         <v>3</v>
@@ -1377,10 +1377,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="G15" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.71</v>
       </c>
       <c r="H15" t="n">
         <v>0.93</v>
@@ -1389,7 +1389,7 @@
         <v>0.87</v>
       </c>
       <c r="J15" t="n">
-        <v>0.843</v>
+        <v>0.775</v>
       </c>
       <c r="K15" t="n">
         <v>1</v>
@@ -1440,10 +1440,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="G16" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H16" t="n">
         <v>0.7</v>
@@ -1452,7 +1452,7 @@
         <v>0.87</v>
       </c>
       <c r="J16" t="n">
-        <v>0.8165</v>
+        <v>0.745</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -1503,10 +1503,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.9</v>
+        <v>0.78</v>
       </c>
       <c r="G17" t="n">
-        <v>0.89</v>
+        <v>0.78</v>
       </c>
       <c r="H17" t="n">
         <v>0.86</v>
@@ -1515,7 +1515,7 @@
         <v>0.84</v>
       </c>
       <c r="J17" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.805</v>
       </c>
       <c r="K17" t="n">
         <v>1</v>
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="G18" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="H18" t="n">
         <v>0.61</v>
@@ -1578,7 +1578,7 @@
         <v>0.84</v>
       </c>
       <c r="J18" t="n">
-        <v>0.8395</v>
+        <v>0.7615</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>0.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H19" t="n">
         <v>0.29</v>
@@ -1641,7 +1641,7 @@
         <v>0.65</v>
       </c>
       <c r="J19" t="n">
-        <v>0.76</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
@@ -1755,10 +1755,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>0.7</v>
@@ -1767,7 +1767,7 @@
         <v>0.65</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.8875</v>
       </c>
       <c r="K21" t="n">
         <v>2</v>
@@ -1818,10 +1818,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>0.93</v>
@@ -1830,7 +1830,7 @@
         <v>0.65</v>
       </c>
       <c r="J22" t="n">
-        <v>0.9075</v>
+        <v>0.9335</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
@@ -1881,10 +1881,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="G23" t="n">
-        <v>0.73</v>
+        <v>0.64</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
@@ -1893,7 +1893,7 @@
         <v>0.84</v>
       </c>
       <c r="J23" t="n">
-        <v>0.8005</v>
+        <v>0.739</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
@@ -1944,10 +1944,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.77</v>
+        <v>0.66</v>
       </c>
       <c r="G24" t="n">
-        <v>0.76</v>
+        <v>0.67</v>
       </c>
       <c r="H24" t="n">
         <v>0.78</v>
@@ -1956,7 +1956,7 @@
         <v>0.84</v>
       </c>
       <c r="J24" t="n">
-        <v>0.779</v>
+        <v>0.7145</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -2007,10 +2007,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H25" t="n">
         <v>0.51</v>
@@ -2019,7 +2019,7 @@
         <v>0.87</v>
       </c>
       <c r="J25" t="n">
-        <v>0.7524999999999999</v>
+        <v>0.681</v>
       </c>
       <c r="K25" t="n">
         <v>3</v>
@@ -2070,10 +2070,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.78</v>
+        <v>0.95</v>
       </c>
       <c r="G26" t="n">
-        <v>0.78</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H26" t="n">
         <v>0.7</v>
@@ -2082,7 +2082,7 @@
         <v>0.65</v>
       </c>
       <c r="J26" t="n">
-        <v>0.7445000000000001</v>
+        <v>0.8515</v>
       </c>
       <c r="K26" t="n">
         <v>2</v>
@@ -2133,10 +2133,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.73</v>
+        <v>0.9</v>
       </c>
       <c r="G27" t="n">
-        <v>0.73</v>
+        <v>0.9</v>
       </c>
       <c r="H27" t="n">
         <v>0.93</v>
@@ -2145,7 +2145,7 @@
         <v>0.65</v>
       </c>
       <c r="J27" t="n">
-        <v>0.758</v>
+        <v>0.8685</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -2196,10 +2196,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="H28" t="n">
         <v>0.86</v>
@@ -2208,7 +2208,7 @@
         <v>0.65</v>
       </c>
       <c r="J28" t="n">
-        <v>0.718</v>
+        <v>0.8285</v>
       </c>
       <c r="K28" t="n">
         <v>3</v>
@@ -2259,10 +2259,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
         <v>0.78</v>
@@ -2271,7 +2271,7 @@
         <v>0.65</v>
       </c>
       <c r="J29" t="n">
-        <v>0.871</v>
+        <v>0.9035</v>
       </c>
       <c r="K29" t="n">
         <v>2</v>
@@ -2322,10 +2322,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="G30" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="H30" t="n">
         <v>1</v>
@@ -2334,7 +2334,7 @@
         <v>0.65</v>
       </c>
       <c r="J30" t="n">
-        <v>0.8985</v>
+        <v>0.9345</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
@@ -2385,10 +2385,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="H31" t="n">
         <v>0.78</v>
@@ -2397,7 +2397,7 @@
         <v>0.65</v>
       </c>
       <c r="J31" t="n">
-        <v>0.8385</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
@@ -2448,10 +2448,10 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G32" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
@@ -2460,7 +2460,7 @@
         <v>0.84</v>
       </c>
       <c r="J32" t="n">
-        <v>0.846</v>
+        <v>0.7745</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
@@ -2511,10 +2511,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
       <c r="G33" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="H33" t="n">
         <v>0.78</v>
@@ -2523,7 +2523,7 @@
         <v>0.84</v>
       </c>
       <c r="J33" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.747</v>
       </c>
       <c r="K33" t="n">
         <v>2</v>
@@ -2574,10 +2574,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0.85</v>
+        <v>0.73</v>
       </c>
       <c r="G34" t="n">
-        <v>0.84</v>
+        <v>0.74</v>
       </c>
       <c r="H34" t="n">
         <v>0.51</v>
@@ -2586,7 +2586,7 @@
         <v>0.87</v>
       </c>
       <c r="J34" t="n">
-        <v>0.7815</v>
+        <v>0.7105</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
@@ -2637,10 +2637,10 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>0.83</v>
+        <v>0.98</v>
       </c>
       <c r="G35" t="n">
-        <v>0.82</v>
+        <v>0.98</v>
       </c>
       <c r="H35" t="n">
         <v>0.61</v>
@@ -2649,7 +2649,7 @@
         <v>0.65</v>
       </c>
       <c r="J35" t="n">
-        <v>0.7554999999999999</v>
+        <v>0.8565</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
@@ -2700,10 +2700,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0.79</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G36" t="n">
-        <v>0.79</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H36" t="n">
         <v>0.86</v>
@@ -2712,7 +2712,7 @@
         <v>0.65</v>
       </c>
       <c r="J36" t="n">
-        <v>0.783</v>
+        <v>0.8804999999999999</v>
       </c>
       <c r="K36" t="n">
         <v>1</v>
@@ -2763,10 +2763,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.75</v>
+        <v>0.91</v>
       </c>
       <c r="G37" t="n">
-        <v>0.75</v>
+        <v>0.91</v>
       </c>
       <c r="H37" t="n">
         <v>0.93</v>
@@ -2775,7 +2775,7 @@
         <v>0.65</v>
       </c>
       <c r="J37" t="n">
-        <v>0.771</v>
+        <v>0.875</v>
       </c>
       <c r="K37" t="n">
         <v>2</v>
@@ -2826,10 +2826,10 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="G38" t="n">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="H38" t="n">
         <v>1</v>
@@ -2838,7 +2838,7 @@
         <v>0.84</v>
       </c>
       <c r="J38" t="n">
-        <v>0.836</v>
+        <v>0.768</v>
       </c>
       <c r="K38" t="n">
         <v>1</v>
@@ -2889,10 +2889,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="G39" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H39" t="n">
         <v>0.73</v>
@@ -2901,7 +2901,7 @@
         <v>0.84</v>
       </c>
       <c r="J39" t="n">
-        <v>0.795</v>
+        <v>0.727</v>
       </c>
       <c r="K39" t="n">
         <v>2</v>
@@ -2952,10 +2952,10 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0.83</v>
+        <v>0.71</v>
       </c>
       <c r="G40" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="H40" t="n">
         <v>0.38</v>
@@ -2964,7 +2964,7 @@
         <v>0.84</v>
       </c>
       <c r="J40" t="n">
-        <v>0.738</v>
+        <v>0.667</v>
       </c>
       <c r="K40" t="n">
         <v>3</v>
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="G41" t="n">
-        <v>0.79</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H41" t="n">
         <v>0.78</v>
@@ -3027,7 +3027,7 @@
         <v>0.84</v>
       </c>
       <c r="J41" t="n">
-        <v>0.7955</v>
+        <v>0.7275</v>
       </c>
       <c r="K41" t="n">
         <v>3</v>
@@ -3078,10 +3078,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0.82</v>
+        <v>0.7</v>
       </c>
       <c r="G42" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.71</v>
       </c>
       <c r="H42" t="n">
         <v>1</v>
@@ -3090,7 +3090,7 @@
         <v>0.84</v>
       </c>
       <c r="J42" t="n">
-        <v>0.8555</v>
+        <v>0.7845</v>
       </c>
       <c r="K42" t="n">
         <v>1</v>
@@ -3141,10 +3141,10 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="G43" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H43" t="n">
         <v>0.78</v>
@@ -3153,7 +3153,7 @@
         <v>0.87</v>
       </c>
       <c r="J43" t="n">
-        <v>0.8325</v>
+        <v>0.761</v>
       </c>
       <c r="K43" t="n">
         <v>2</v>
@@ -3204,10 +3204,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="G44" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="H44" t="n">
         <v>0.86</v>
@@ -3216,7 +3216,7 @@
         <v>0.84</v>
       </c>
       <c r="J44" t="n">
-        <v>0.7465000000000001</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="K44" t="n">
         <v>1</v>
@@ -3267,10 +3267,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="G45" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="H45" t="n">
         <v>0.61</v>
@@ -3279,7 +3279,7 @@
         <v>0.84</v>
       </c>
       <c r="J45" t="n">
-        <v>0.7225</v>
+        <v>0.6575</v>
       </c>
       <c r="K45" t="n">
         <v>2</v>
@@ -3330,10 +3330,10 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>0.76</v>
+        <v>0.66</v>
       </c>
       <c r="G46" t="n">
-        <v>0.76</v>
+        <v>0.66</v>
       </c>
       <c r="H46" t="n">
         <v>0.29</v>
@@ -3342,7 +3342,7 @@
         <v>0.65</v>
       </c>
       <c r="J46" t="n">
-        <v>0.6495</v>
+        <v>0.5845</v>
       </c>
       <c r="K46" t="n">
         <v>3</v>
@@ -3393,10 +3393,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>0.61</v>
+        <v>0.85</v>
       </c>
       <c r="G47" t="n">
-        <v>0.61</v>
+        <v>0.85</v>
       </c>
       <c r="H47" t="n">
         <v>0.51</v>
@@ -3405,7 +3405,7 @@
         <v>0.65</v>
       </c>
       <c r="J47" t="n">
-        <v>0.596</v>
+        <v>0.752</v>
       </c>
       <c r="K47" t="n">
         <v>3</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="G48" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="H48" t="n">
         <v>0.78</v>
@@ -3468,7 +3468,7 @@
         <v>0.65</v>
       </c>
       <c r="J48" t="n">
-        <v>0.6175</v>
+        <v>0.7735</v>
       </c>
       <c r="K48" t="n">
         <v>2</v>
@@ -3519,10 +3519,10 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="G49" t="n">
-        <v>0.51</v>
+        <v>0.75</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
@@ -3531,7 +3531,7 @@
         <v>0.65</v>
       </c>
       <c r="J49" t="n">
-        <v>0.626</v>
+        <v>0.785</v>
       </c>
       <c r="K49" t="n">
         <v>1</v>
@@ -3582,10 +3582,10 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>0.71</v>
+        <v>0.61</v>
       </c>
       <c r="G50" t="n">
-        <v>0.71</v>
+        <v>0.62</v>
       </c>
       <c r="H50" t="n">
         <v>0.93</v>
@@ -3594,7 +3594,7 @@
         <v>0.87</v>
       </c>
       <c r="J50" t="n">
-        <v>0.778</v>
+        <v>0.7165</v>
       </c>
       <c r="K50" t="n">
         <v>2</v>
@@ -3645,10 +3645,10 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="G51" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="H51" t="n">
         <v>0.86</v>
@@ -3657,7 +3657,7 @@
         <v>0.87</v>
       </c>
       <c r="J51" t="n">
-        <v>0.79</v>
+        <v>0.722</v>
       </c>
       <c r="K51" t="n">
         <v>1</v>
@@ -3708,10 +3708,10 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="G52" t="n">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="H52" t="n">
         <v>0.61</v>
@@ -3720,7 +3720,7 @@
         <v>0.87</v>
       </c>
       <c r="J52" t="n">
-        <v>0.7595</v>
+        <v>0.6945</v>
       </c>
       <c r="K52" t="n">
         <v>3</v>
@@ -3771,10 +3771,10 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.78</v>
+        <v>0.67</v>
       </c>
       <c r="G53" t="n">
-        <v>0.78</v>
+        <v>0.68</v>
       </c>
       <c r="H53" t="n">
         <v>0.83</v>
@@ -3783,7 +3783,7 @@
         <v>0.84</v>
       </c>
       <c r="J53" t="n">
-        <v>0.799</v>
+        <v>0.731</v>
       </c>
       <c r="K53" t="n">
         <v>1</v>
@@ -3834,10 +3834,10 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G54" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H54" t="n">
         <v>0.51</v>
@@ -3846,7 +3846,7 @@
         <v>0.84</v>
       </c>
       <c r="J54" t="n">
-        <v>0.748</v>
+        <v>0.68</v>
       </c>
       <c r="K54" t="n">
         <v>2</v>
@@ -3897,10 +3897,10 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
       <c r="G55" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="H55" t="n">
         <v>0.06</v>
@@ -3909,7 +3909,7 @@
         <v>0.65</v>
       </c>
       <c r="J55" t="n">
-        <v>0.6425</v>
+        <v>0.5745</v>
       </c>
       <c r="K55" t="n">
         <v>3</v>
@@ -3960,10 +3960,10 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="G56" t="n">
-        <v>0.51</v>
+        <v>0.43</v>
       </c>
       <c r="H56" t="n">
         <v>0.51</v>
@@ -3972,7 +3972,7 @@
         <v>0.84</v>
       </c>
       <c r="J56" t="n">
-        <v>0.5565</v>
+        <v>0.5044999999999999</v>
       </c>
       <c r="K56" t="n">
         <v>3</v>
@@ -4023,10 +4023,10 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0.55</v>
+        <v>0.47</v>
       </c>
       <c r="G57" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="H57" t="n">
         <v>0.92</v>
@@ -4035,7 +4035,7 @@
         <v>0.84</v>
       </c>
       <c r="J57" t="n">
-        <v>0.671</v>
+        <v>0.619</v>
       </c>
       <c r="K57" t="n">
         <v>1</v>
@@ -4086,10 +4086,10 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="G58" t="n">
-        <v>0.61</v>
+        <v>0.53</v>
       </c>
       <c r="H58" t="n">
         <v>0.73</v>
@@ -4098,7 +4098,7 @@
         <v>0.84</v>
       </c>
       <c r="J58" t="n">
-        <v>0.6685</v>
+        <v>0.6135</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
@@ -4149,10 +4149,10 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>0.35</v>
+        <v>0.72</v>
       </c>
       <c r="G59" t="n">
-        <v>0.36</v>
+        <v>0.73</v>
       </c>
       <c r="H59" t="n">
         <v>0.51</v>
@@ -4161,7 +4161,7 @@
         <v>0.65</v>
       </c>
       <c r="J59" t="n">
-        <v>0.4305</v>
+        <v>0.671</v>
       </c>
       <c r="K59" t="n">
         <v>2</v>
@@ -4212,10 +4212,10 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0.28</v>
+        <v>0.66</v>
       </c>
       <c r="G60" t="n">
-        <v>0.29</v>
+        <v>0.66</v>
       </c>
       <c r="H60" t="n">
         <v>0.83</v>
@@ -4224,7 +4224,7 @@
         <v>0.65</v>
       </c>
       <c r="J60" t="n">
-        <v>0.449</v>
+        <v>0.6925</v>
       </c>
       <c r="K60" t="n">
         <v>1</v>
@@ -4275,10 +4275,10 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0.2</v>
+        <v>0.59</v>
       </c>
       <c r="G61" t="n">
-        <v>0.22</v>
+        <v>0.6</v>
       </c>
       <c r="H61" t="n">
         <v>0.92</v>
@@ -4287,7 +4287,7 @@
         <v>0.65</v>
       </c>
       <c r="J61" t="n">
-        <v>0.4185</v>
+        <v>0.6685</v>
       </c>
       <c r="K61" t="n">
         <v>3</v>
@@ -4338,10 +4338,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>0.67</v>
+        <v>0.89</v>
       </c>
       <c r="G62" t="n">
-        <v>0.67</v>
+        <v>0.89</v>
       </c>
       <c r="H62" t="n">
         <v>0.51</v>
@@ -4350,7 +4350,7 @@
         <v>0.65</v>
       </c>
       <c r="J62" t="n">
-        <v>0.635</v>
+        <v>0.778</v>
       </c>
       <c r="K62" t="n">
         <v>3</v>
@@ -4401,10 +4401,10 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.61</v>
+        <v>0.84</v>
       </c>
       <c r="G63" t="n">
-        <v>0.62</v>
+        <v>0.84</v>
       </c>
       <c r="H63" t="n">
         <v>0.78</v>
@@ -4413,7 +4413,7 @@
         <v>0.65</v>
       </c>
       <c r="J63" t="n">
-        <v>0.6535</v>
+        <v>0.7995</v>
       </c>
       <c r="K63" t="n">
         <v>2</v>
@@ -4464,10 +4464,10 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="G64" t="n">
-        <v>0.57</v>
+        <v>0.79</v>
       </c>
       <c r="H64" t="n">
         <v>1</v>
@@ -4476,7 +4476,7 @@
         <v>0.65</v>
       </c>
       <c r="J64" t="n">
-        <v>0.665</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="K64" t="n">
         <v>1</v>
@@ -4527,10 +4527,10 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.53</v>
+        <v>0.45</v>
       </c>
       <c r="G65" t="n">
-        <v>0.54</v>
+        <v>0.46</v>
       </c>
       <c r="H65" t="n">
         <v>0.92</v>
@@ -4539,7 +4539,7 @@
         <v>0.84</v>
       </c>
       <c r="J65" t="n">
-        <v>0.658</v>
+        <v>0.606</v>
       </c>
       <c r="K65" t="n">
         <v>2</v>
@@ -4590,10 +4590,10 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="G66" t="n">
-        <v>0.59</v>
+        <v>0.51</v>
       </c>
       <c r="H66" t="n">
         <v>0.83</v>
@@ -4602,7 +4602,7 @@
         <v>0.87</v>
       </c>
       <c r="J66" t="n">
-        <v>0.677</v>
+        <v>0.625</v>
       </c>
       <c r="K66" t="n">
         <v>1</v>
@@ -4653,10 +4653,10 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.63</v>
+        <v>0.54</v>
       </c>
       <c r="G67" t="n">
-        <v>0.63</v>
+        <v>0.55</v>
       </c>
       <c r="H67" t="n">
         <v>0.51</v>
@@ -4665,7 +4665,7 @@
         <v>0.87</v>
       </c>
       <c r="J67" t="n">
-        <v>0.642</v>
+        <v>0.587</v>
       </c>
       <c r="K67" t="n">
         <v>3</v>
@@ -4716,10 +4716,10 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0.41</v>
+        <v>0.73</v>
       </c>
       <c r="G68" t="n">
-        <v>0.42</v>
+        <v>0.73</v>
       </c>
       <c r="H68" t="n">
         <v>0.46</v>
@@ -4728,7 +4728,7 @@
         <v>0.65</v>
       </c>
       <c r="J68" t="n">
-        <v>0.4595</v>
+        <v>0.664</v>
       </c>
       <c r="K68" t="n">
         <v>3</v>
@@ -4779,10 +4779,10 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.34</v>
+        <v>0.67</v>
       </c>
       <c r="G69" t="n">
-        <v>0.36</v>
+        <v>0.67</v>
       </c>
       <c r="H69" t="n">
         <v>0.8100000000000001</v>
@@ -4791,7 +4791,7 @@
         <v>0.65</v>
       </c>
       <c r="J69" t="n">
-        <v>0.4875</v>
+        <v>0.695</v>
       </c>
       <c r="K69" t="n">
         <v>1</v>
@@ -4842,10 +4842,10 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.27</v>
+        <v>0.61</v>
       </c>
       <c r="G70" t="n">
-        <v>0.29</v>
+        <v>0.61</v>
       </c>
       <c r="H70" t="n">
         <v>0.91</v>
@@ -4854,7 +4854,7 @@
         <v>0.65</v>
       </c>
       <c r="J70" t="n">
-        <v>0.462</v>
+        <v>0.676</v>
       </c>
       <c r="K70" t="n">
         <v>2</v>
@@ -4905,10 +4905,10 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="G71" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="H71" t="n">
         <v>0.86</v>
@@ -4917,7 +4917,7 @@
         <v>0.84</v>
       </c>
       <c r="J71" t="n">
-        <v>0.7335</v>
+        <v>0.675</v>
       </c>
       <c r="K71" t="n">
         <v>1</v>
@@ -4968,10 +4968,10 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>0.71</v>
+        <v>0.61</v>
       </c>
       <c r="G72" t="n">
-        <v>0.71</v>
+        <v>0.62</v>
       </c>
       <c r="H72" t="n">
         <v>0.61</v>
@@ -4980,7 +4980,7 @@
         <v>0.87</v>
       </c>
       <c r="J72" t="n">
-        <v>0.714</v>
+        <v>0.6525</v>
       </c>
       <c r="K72" t="n">
         <v>2</v>
@@ -5031,10 +5031,10 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="G73" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="H73" t="n">
         <v>0.29</v>
@@ -5043,7 +5043,7 @@
         <v>0.65</v>
       </c>
       <c r="J73" t="n">
-        <v>0.643</v>
+        <v>0.575</v>
       </c>
       <c r="K73" t="n">
         <v>3</v>
@@ -5094,10 +5094,10 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
       <c r="G74" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="H74" t="n">
         <v>1</v>
@@ -5106,7 +5106,7 @@
         <v>0.84</v>
       </c>
       <c r="J74" t="n">
-        <v>0.5765</v>
+        <v>0.5345</v>
       </c>
       <c r="K74" t="n">
         <v>1</v>
@@ -5157,10 +5157,10 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="G75" t="n">
-        <v>0.44</v>
+        <v>0.38</v>
       </c>
       <c r="H75" t="n">
         <v>0.78</v>
@@ -5169,7 +5169,7 @@
         <v>0.84</v>
       </c>
       <c r="J75" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.526</v>
       </c>
       <c r="K75" t="n">
         <v>2</v>
@@ -5220,10 +5220,10 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>0.49</v>
+        <v>0.42</v>
       </c>
       <c r="G76" t="n">
-        <v>0.5</v>
+        <v>0.43</v>
       </c>
       <c r="H76" t="n">
         <v>0.51</v>
@@ -5232,7 +5232,7 @@
         <v>0.87</v>
       </c>
       <c r="J76" t="n">
-        <v>0.5545</v>
+        <v>0.509</v>
       </c>
       <c r="K76" t="n">
         <v>3</v>
@@ -5283,10 +5283,10 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="G77" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="H77" t="n">
         <v>0.61</v>
@@ -5295,7 +5295,7 @@
         <v>0.65</v>
       </c>
       <c r="J77" t="n">
-        <v>0.6745</v>
+        <v>0.8045</v>
       </c>
       <c r="K77" t="n">
         <v>3</v>
@@ -5346,10 +5346,10 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.65</v>
+        <v>0.86</v>
       </c>
       <c r="G78" t="n">
-        <v>0.65</v>
+        <v>0.86</v>
       </c>
       <c r="H78" t="n">
         <v>0.86</v>
@@ -5358,7 +5358,7 @@
         <v>0.65</v>
       </c>
       <c r="J78" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.8285</v>
       </c>
       <c r="K78" t="n">
         <v>1</v>
@@ -5409,10 +5409,10 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.61</v>
+        <v>0.82</v>
       </c>
       <c r="G79" t="n">
-        <v>0.61</v>
+        <v>0.82</v>
       </c>
       <c r="H79" t="n">
         <v>0.93</v>
@@ -5421,7 +5421,7 @@
         <v>0.65</v>
       </c>
       <c r="J79" t="n">
-        <v>0.68</v>
+        <v>0.8165</v>
       </c>
       <c r="K79" t="n">
         <v>2</v>
@@ -5472,10 +5472,10 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.37</v>
+        <v>0.71</v>
       </c>
       <c r="G80" t="n">
-        <v>0.38</v>
+        <v>0.71</v>
       </c>
       <c r="H80" t="n">
         <v>0.61</v>
@@ -5484,7 +5484,7 @@
         <v>0.65</v>
       </c>
       <c r="J80" t="n">
-        <v>0.4635</v>
+        <v>0.681</v>
       </c>
       <c r="K80" t="n">
         <v>2</v>
@@ -5535,10 +5535,10 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>0.29</v>
+        <v>0.64</v>
       </c>
       <c r="G81" t="n">
-        <v>0.31</v>
+        <v>0.65</v>
       </c>
       <c r="H81" t="n">
         <v>0.86</v>
@@ -5547,7 +5547,7 @@
         <v>0.65</v>
       </c>
       <c r="J81" t="n">
-        <v>0.465</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="K81" t="n">
         <v>1</v>
@@ -5598,10 +5598,10 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>0.21</v>
+        <v>0.58</v>
       </c>
       <c r="G82" t="n">
-        <v>0.23</v>
+        <v>0.58</v>
       </c>
       <c r="H82" t="n">
         <v>0.93</v>
@@ -5610,7 +5610,7 @@
         <v>0.65</v>
       </c>
       <c r="J82" t="n">
-        <v>0.427</v>
+        <v>0.6605</v>
       </c>
       <c r="K82" t="n">
         <v>3</v>
@@ -5661,10 +5661,10 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="G83" t="n">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="H83" t="n">
         <v>0.85</v>
@@ -5673,7 +5673,7 @@
         <v>0.77</v>
       </c>
       <c r="J83" t="n">
-        <v>0.5004999999999999</v>
+        <v>0.4645</v>
       </c>
       <c r="K83" t="n">
         <v>1</v>
@@ -5724,10 +5724,10 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="G84" t="n">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="H84" t="n">
         <v>0.67</v>
@@ -5736,7 +5736,7 @@
         <v>0.84</v>
       </c>
       <c r="J84" t="n">
-        <v>0.4975</v>
+        <v>0.4585</v>
       </c>
       <c r="K84" t="n">
         <v>2</v>
@@ -5787,10 +5787,10 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G85" t="n">
-        <v>0.41</v>
+        <v>0.35</v>
       </c>
       <c r="H85" t="n">
         <v>0.45</v>
@@ -5799,7 +5799,7 @@
         <v>0.84</v>
       </c>
       <c r="J85" t="n">
-        <v>0.4795</v>
+        <v>0.4375</v>
       </c>
       <c r="K85" t="n">
         <v>3</v>
@@ -5850,10 +5850,10 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="G86" t="n">
-        <v>0.29</v>
+        <v>0.24</v>
       </c>
       <c r="H86" t="n">
         <v>0.73</v>
@@ -5862,7 +5862,7 @@
         <v>0.84</v>
       </c>
       <c r="J86" t="n">
-        <v>0.4575</v>
+        <v>0.425</v>
       </c>
       <c r="K86" t="n">
         <v>1</v>
@@ -5913,10 +5913,10 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
       <c r="G87" t="n">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="H87" t="n">
         <v>0.51</v>
@@ -5925,7 +5925,7 @@
         <v>0.84</v>
       </c>
       <c r="J87" t="n">
-        <v>0.4395</v>
+        <v>0.404</v>
       </c>
       <c r="K87" t="n">
         <v>2</v>
@@ -5976,10 +5976,10 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="G88" t="n">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="H88" t="n">
         <v>0.23</v>
@@ -5988,7 +5988,7 @@
         <v>0.74</v>
       </c>
       <c r="J88" t="n">
-        <v>0.3945</v>
+        <v>0.3555</v>
       </c>
       <c r="K88" t="n">
         <v>3</v>
@@ -6039,10 +6039,10 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>0.57</v>
+        <v>0.49</v>
       </c>
       <c r="G89" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="H89" t="n">
         <v>0.93</v>
@@ -6051,7 +6051,7 @@
         <v>0.84</v>
       </c>
       <c r="J89" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.634</v>
       </c>
       <c r="K89" t="n">
         <v>1</v>
@@ -6102,10 +6102,10 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.6</v>
+        <v>0.51</v>
       </c>
       <c r="G90" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="H90" t="n">
         <v>0.78</v>
@@ -6114,7 +6114,7 @@
         <v>0.84</v>
       </c>
       <c r="J90" t="n">
-        <v>0.6755</v>
+        <v>0.617</v>
       </c>
       <c r="K90" t="n">
         <v>2</v>
@@ -6165,10 +6165,10 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0.63</v>
+        <v>0.54</v>
       </c>
       <c r="G91" t="n">
-        <v>0.63</v>
+        <v>0.55</v>
       </c>
       <c r="H91" t="n">
         <v>0.61</v>
@@ -6177,7 +6177,7 @@
         <v>0.84</v>
       </c>
       <c r="J91" t="n">
-        <v>0.6575</v>
+        <v>0.6025</v>
       </c>
       <c r="K91" t="n">
         <v>3</v>
@@ -6228,10 +6228,10 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="G92" t="n">
-        <v>0.57</v>
+        <v>0.49</v>
       </c>
       <c r="H92" t="n">
         <v>0.45</v>
@@ -6240,7 +6240,7 @@
         <v>0.87</v>
       </c>
       <c r="J92" t="n">
-        <v>0.588</v>
+        <v>0.536</v>
       </c>
       <c r="K92" t="n">
         <v>2</v>
@@ -6291,10 +6291,10 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="G93" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="H93" t="n">
         <v>1</v>
@@ -6303,7 +6303,7 @@
         <v>0.84</v>
       </c>
       <c r="J93" t="n">
-        <v>0.635</v>
+        <v>0.5895</v>
       </c>
       <c r="K93" t="n">
         <v>1</v>
@@ -6354,10 +6354,10 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="G94" t="n">
-        <v>0.38</v>
+        <v>0.32</v>
       </c>
       <c r="H94" t="n">
         <v>0.45</v>
@@ -6366,7 +6366,7 @@
         <v>0.71</v>
       </c>
       <c r="J94" t="n">
-        <v>0.4405</v>
+        <v>0.4015</v>
       </c>
       <c r="K94" t="n">
         <v>3</v>
@@ -6417,10 +6417,10 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="G95" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="H95" t="n">
         <v>0.86</v>
@@ -6429,7 +6429,7 @@
         <v>0.77</v>
       </c>
       <c r="J95" t="n">
-        <v>0.512</v>
+        <v>0.4765</v>
       </c>
       <c r="K95" t="n">
         <v>1</v>
@@ -6480,10 +6480,10 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="G96" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="H96" t="n">
         <v>0.7</v>
@@ -6492,7 +6492,7 @@
         <v>0.77</v>
       </c>
       <c r="J96" t="n">
-        <v>0.503</v>
+        <v>0.464</v>
       </c>
       <c r="K96" t="n">
         <v>2</v>
@@ -6543,10 +6543,10 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0.41</v>
+        <v>0.34</v>
       </c>
       <c r="G97" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="H97" t="n">
         <v>0.51</v>
@@ -6555,7 +6555,7 @@
         <v>0.77</v>
       </c>
       <c r="J97" t="n">
-        <v>0.4875</v>
+        <v>0.4455</v>
       </c>
       <c r="K97" t="n">
         <v>3</v>
@@ -6606,10 +6606,10 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0.38</v>
+        <v>0.32</v>
       </c>
       <c r="G98" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="H98" t="n">
         <v>0.76</v>
@@ -6618,7 +6618,7 @@
         <v>0.84</v>
       </c>
       <c r="J98" t="n">
-        <v>0.5285</v>
+        <v>0.4895</v>
       </c>
       <c r="K98" t="n">
         <v>1</v>
@@ -6669,10 +6669,10 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="G99" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="H99" t="n">
         <v>0.5600000000000001</v>
@@ -6681,7 +6681,7 @@
         <v>0.84</v>
       </c>
       <c r="J99" t="n">
-        <v>0.5145</v>
+        <v>0.4725</v>
       </c>
       <c r="K99" t="n">
         <v>2</v>
@@ -6732,10 +6732,10 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="G100" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="H100" t="n">
         <v>0.32</v>
@@ -6744,7 +6744,7 @@
         <v>0.74</v>
       </c>
       <c r="J100" t="n">
-        <v>0.4775</v>
+        <v>0.432</v>
       </c>
       <c r="K100" t="n">
         <v>3</v>
@@ -6795,10 +6795,10 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="G101" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H101" t="n">
         <v>0.86</v>
@@ -6807,7 +6807,7 @@
         <v>0.84</v>
       </c>
       <c r="J101" t="n">
-        <v>0.7205</v>
+        <v>0.659</v>
       </c>
       <c r="K101" t="n">
         <v>1</v>
@@ -6858,10 +6858,10 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="G102" t="n">
-        <v>0.68</v>
+        <v>0.59</v>
       </c>
       <c r="H102" t="n">
         <v>0.7</v>
@@ -6870,7 +6870,7 @@
         <v>0.87</v>
       </c>
       <c r="J102" t="n">
-        <v>0.7095</v>
+        <v>0.651</v>
       </c>
       <c r="K102" t="n">
         <v>2</v>
@@ -6921,10 +6921,10 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="G103" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="H103" t="n">
         <v>0.51</v>
@@ -6933,7 +6933,7 @@
         <v>0.87</v>
       </c>
       <c r="J103" t="n">
-        <v>0.6875</v>
+        <v>0.626</v>
       </c>
       <c r="K103" t="n">
         <v>3</v>
@@ -6984,10 +6984,10 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="G104" t="n">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="H104" t="n">
         <v>0</v>
@@ -6996,10 +6996,10 @@
         <v>0.31</v>
       </c>
       <c r="J104" t="n">
-        <v>0.0465</v>
+        <v>0.3945</v>
       </c>
       <c r="K104" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L104" t="n">
         <v>3000</v>
@@ -7047,10 +7047,10 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
+        <v>0.43</v>
       </c>
       <c r="G105" t="n">
-        <v>0</v>
+        <v>0.44</v>
       </c>
       <c r="H105" t="n">
         <v>0.06</v>
@@ -7059,10 +7059,10 @@
         <v>0.65</v>
       </c>
       <c r="J105" t="n">
-        <v>0.1095</v>
+        <v>0.3925</v>
       </c>
       <c r="K105" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L105" t="n">
         <v>3000</v>
@@ -7110,10 +7110,10 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G106" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="H106" t="n">
         <v>0.63</v>
@@ -7122,7 +7122,7 @@
         <v>0.65</v>
       </c>
       <c r="J106" t="n">
-        <v>0.2235</v>
+        <v>0.4255</v>
       </c>
       <c r="K106" t="n">
         <v>1</v>
@@ -7173,10 +7173,10 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>0.68</v>
+        <v>0.59</v>
       </c>
       <c r="G107" t="n">
-        <v>0.68</v>
+        <v>0.59</v>
       </c>
       <c r="H107" t="n">
         <v>0.78</v>
@@ -7185,7 +7185,7 @@
         <v>0.87</v>
       </c>
       <c r="J107" t="n">
-        <v>0.7285</v>
+        <v>0.67</v>
       </c>
       <c r="K107" t="n">
         <v>3</v>
@@ -7236,10 +7236,10 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="G108" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="H108" t="n">
         <v>1</v>
@@ -7248,7 +7248,7 @@
         <v>0.87</v>
       </c>
       <c r="J108" t="n">
-        <v>0.805</v>
+        <v>0.74</v>
       </c>
       <c r="K108" t="n">
         <v>1</v>
@@ -7299,10 +7299,10 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0.78</v>
+        <v>0.67</v>
       </c>
       <c r="G109" t="n">
-        <v>0.77</v>
+        <v>0.67</v>
       </c>
       <c r="H109" t="n">
         <v>0.78</v>
@@ -7311,7 +7311,7 @@
         <v>0.87</v>
       </c>
       <c r="J109" t="n">
-        <v>0.79</v>
+        <v>0.722</v>
       </c>
       <c r="K109" t="n">
         <v>2</v>
@@ -7362,10 +7362,10 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="G110" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="H110" t="n">
         <v>0.83</v>
@@ -7374,7 +7374,7 @@
         <v>0.87</v>
       </c>
       <c r="J110" t="n">
-        <v>0.5925</v>
+        <v>0.547</v>
       </c>
       <c r="K110" t="n">
         <v>3</v>
@@ -7425,10 +7425,10 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0.53</v>
+        <v>0.45</v>
       </c>
       <c r="G111" t="n">
-        <v>0.54</v>
+        <v>0.46</v>
       </c>
       <c r="H111" t="n">
         <v>0.83</v>
@@ -7437,7 +7437,7 @@
         <v>0.87</v>
       </c>
       <c r="J111" t="n">
-        <v>0.6445</v>
+        <v>0.5925</v>
       </c>
       <c r="K111" t="n">
         <v>1</v>
@@ -7488,10 +7488,10 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0.57</v>
+        <v>0.49</v>
       </c>
       <c r="G112" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="H112" t="n">
         <v>0.63</v>
@@ -7500,7 +7500,7 @@
         <v>0.87</v>
       </c>
       <c r="J112" t="n">
-        <v>0.6304999999999999</v>
+        <v>0.5785</v>
       </c>
       <c r="K112" t="n">
         <v>2</v>
@@ -7566,7 +7566,7 @@
         <v>0.888</v>
       </c>
       <c r="K113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L113" t="n">
         <v>2200</v>
@@ -7614,10 +7614,10 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="G114" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="H114" t="n">
         <v>0.85</v>
@@ -7626,10 +7626,10 @@
         <v>0.77</v>
       </c>
       <c r="J114" t="n">
-        <v>0.8995</v>
+        <v>0.9355</v>
       </c>
       <c r="K114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L114" t="n">
         <v>2200</v>
@@ -7677,10 +7677,10 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>0.87</v>
+        <v>1</v>
       </c>
       <c r="G115" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="H115" t="n">
         <v>0.93</v>
@@ -7689,10 +7689,10 @@
         <v>0.77</v>
       </c>
       <c r="J115" t="n">
-        <v>0.8635</v>
+        <v>0.9515</v>
       </c>
       <c r="K115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L115" t="n">
         <v>2200</v>
@@ -7740,10 +7740,10 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="G116" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H116" t="n">
         <v>0.51</v>
@@ -7752,10 +7752,10 @@
         <v>0.77</v>
       </c>
       <c r="J116" t="n">
-        <v>0.8575</v>
+        <v>0.8675</v>
       </c>
       <c r="K116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L116" t="n">
         <v>1800</v>
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="G117" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="H117" t="n">
         <v>0.78</v>
@@ -7815,10 +7815,10 @@
         <v>0.77</v>
       </c>
       <c r="J117" t="n">
-        <v>0.8725000000000001</v>
+        <v>0.9215</v>
       </c>
       <c r="K117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L117" t="n">
         <v>1800</v>
@@ -7866,10 +7866,10 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="G118" t="n">
-        <v>0.84</v>
+        <v>1</v>
       </c>
       <c r="H118" t="n">
         <v>0.93</v>
@@ -7878,10 +7878,10 @@
         <v>0.77</v>
       </c>
       <c r="J118" t="n">
-        <v>0.8505</v>
+        <v>0.9515</v>
       </c>
       <c r="K118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L118" t="n">
         <v>1800</v>
@@ -7929,10 +7929,10 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="G119" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="H119" t="n">
         <v>0.5600000000000001</v>
@@ -7941,10 +7941,10 @@
         <v>0.77</v>
       </c>
       <c r="J119" t="n">
-        <v>0.861</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="K119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L119" t="n">
         <v>1700</v>
@@ -7992,10 +7992,10 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="G120" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H120" t="n">
         <v>0.93</v>
@@ -8004,7 +8004,7 @@
         <v>0.77</v>
       </c>
       <c r="J120" t="n">
-        <v>0.8865</v>
+        <v>0.9515</v>
       </c>
       <c r="K120" t="n">
         <v>1</v>
@@ -8055,10 +8055,10 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="G121" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="H121" t="n">
         <v>0.76</v>
@@ -8067,10 +8067,10 @@
         <v>0.77</v>
       </c>
       <c r="J121" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.9175</v>
       </c>
       <c r="K121" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L121" t="n">
         <v>1700</v>
@@ -8118,10 +8118,10 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="G122" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="H122" t="n">
         <v>0.61</v>
@@ -8130,7 +8130,7 @@
         <v>0.77</v>
       </c>
       <c r="J122" t="n">
-        <v>0.462</v>
+        <v>0.4265</v>
       </c>
       <c r="K122" t="n">
         <v>3</v>
@@ -8181,10 +8181,10 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="G123" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="H123" t="n">
         <v>1</v>
@@ -8193,7 +8193,7 @@
         <v>0.84</v>
       </c>
       <c r="J123" t="n">
-        <v>0.6025</v>
+        <v>0.5635</v>
       </c>
       <c r="K123" t="n">
         <v>1</v>
@@ -8244,10 +8244,10 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0.52</v>
+        <v>0.45</v>
       </c>
       <c r="G124" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="H124" t="n">
         <v>0.51</v>
@@ -8256,7 +8256,7 @@
         <v>0.84</v>
       </c>
       <c r="J124" t="n">
-        <v>0.5695</v>
+        <v>0.524</v>
       </c>
       <c r="K124" t="n">
         <v>2</v>
@@ -8307,10 +8307,10 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0.77</v>
+        <v>0.98</v>
       </c>
       <c r="G125" t="n">
-        <v>0.77</v>
+        <v>0.97</v>
       </c>
       <c r="H125" t="n">
         <v>0.51</v>
@@ -8319,7 +8319,7 @@
         <v>0.65</v>
       </c>
       <c r="J125" t="n">
-        <v>0.7</v>
+        <v>0.833</v>
       </c>
       <c r="K125" t="n">
         <v>2</v>
@@ -8370,10 +8370,10 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="G126" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H126" t="n">
         <v>0.93</v>
@@ -8382,7 +8382,7 @@
         <v>0.65</v>
       </c>
       <c r="J126" t="n">
-        <v>0.732</v>
+        <v>0.875</v>
       </c>
       <c r="K126" t="n">
         <v>1</v>
@@ -8433,10 +8433,10 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>0.6</v>
+        <v>0.83</v>
       </c>
       <c r="G127" t="n">
-        <v>0.6</v>
+        <v>0.83</v>
       </c>
       <c r="H127" t="n">
         <v>0.61</v>
@@ -8445,7 +8445,7 @@
         <v>0.65</v>
       </c>
       <c r="J127" t="n">
-        <v>0.6095</v>
+        <v>0.759</v>
       </c>
       <c r="K127" t="n">
         <v>3</v>
@@ -8496,10 +8496,10 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>0.51</v>
+        <v>0.43</v>
       </c>
       <c r="G128" t="n">
-        <v>0.51</v>
+        <v>0.44</v>
       </c>
       <c r="H128" t="n">
         <v>0.86</v>
@@ -8508,7 +8508,7 @@
         <v>0.84</v>
       </c>
       <c r="J128" t="n">
-        <v>0.6294999999999999</v>
+        <v>0.581</v>
       </c>
       <c r="K128" t="n">
         <v>2</v>
@@ -8559,10 +8559,10 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>0.62</v>
+        <v>0.53</v>
       </c>
       <c r="G129" t="n">
-        <v>0.63</v>
+        <v>0.54</v>
       </c>
       <c r="H129" t="n">
         <v>0.15</v>
@@ -8571,7 +8571,7 @@
         <v>0.53</v>
       </c>
       <c r="J129" t="n">
-        <v>0.516</v>
+        <v>0.4575</v>
       </c>
       <c r="K129" t="n">
         <v>3</v>
@@ -8685,10 +8685,10 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>0.55</v>
+        <v>0.46</v>
       </c>
       <c r="G131" t="n">
-        <v>0.55</v>
+        <v>0.47</v>
       </c>
       <c r="H131" t="n">
         <v>0.86</v>
@@ -8697,7 +8697,7 @@
         <v>0.84</v>
       </c>
       <c r="J131" t="n">
-        <v>0.6555</v>
+        <v>0.6005</v>
       </c>
       <c r="K131" t="n">
         <v>2</v>
@@ -8748,10 +8748,10 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>0.67</v>
+        <v>0.57</v>
       </c>
       <c r="G132" t="n">
-        <v>0.67</v>
+        <v>0.58</v>
       </c>
       <c r="H132" t="n">
         <v>0.15</v>
@@ -8760,7 +8760,7 @@
         <v>0.53</v>
       </c>
       <c r="J132" t="n">
-        <v>0.545</v>
+        <v>0.4835</v>
       </c>
       <c r="K132" t="n">
         <v>3</v>
@@ -8874,10 +8874,10 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>0.31</v>
+        <v>0.26</v>
       </c>
       <c r="G134" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="H134" t="n">
         <v>0.76</v>
@@ -8886,7 +8886,7 @@
         <v>0.84</v>
       </c>
       <c r="J134" t="n">
-        <v>0.483</v>
+        <v>0.4505</v>
       </c>
       <c r="K134" t="n">
         <v>3</v>
@@ -8937,10 +8937,10 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="G135" t="n">
-        <v>0.41</v>
+        <v>0.35</v>
       </c>
       <c r="H135" t="n">
         <v>0.93</v>
@@ -8949,7 +8949,7 @@
         <v>0.87</v>
       </c>
       <c r="J135" t="n">
-        <v>0.58</v>
+        <v>0.541</v>
       </c>
       <c r="K135" t="n">
         <v>1</v>
@@ -9000,10 +9000,10 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="G136" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="H136" t="n">
         <v>0.67</v>
@@ -9012,7 +9012,7 @@
         <v>0.87</v>
       </c>
       <c r="J136" t="n">
-        <v>0.5735</v>
+        <v>0.528</v>
       </c>
       <c r="K136" t="n">
         <v>2</v>
@@ -9063,10 +9063,10 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>0.21</v>
+        <v>0.59</v>
       </c>
       <c r="G137" t="n">
-        <v>0.31</v>
+        <v>0.6</v>
       </c>
       <c r="H137" t="n">
         <v>0.51</v>
@@ -9075,7 +9075,7 @@
         <v>0.65</v>
       </c>
       <c r="J137" t="n">
-        <v>0.371</v>
+        <v>0.5865</v>
       </c>
       <c r="K137" t="n">
         <v>2</v>
@@ -9126,10 +9126,10 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>0.13</v>
+        <v>0.54</v>
       </c>
       <c r="G138" t="n">
-        <v>0.24</v>
+        <v>0.54</v>
       </c>
       <c r="H138" t="n">
         <v>0.78</v>
@@ -9138,7 +9138,7 @@
         <v>0.65</v>
       </c>
       <c r="J138" t="n">
-        <v>0.3765</v>
+        <v>0.6045</v>
       </c>
       <c r="K138" t="n">
         <v>1</v>
@@ -9189,10 +9189,10 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>0.06</v>
+        <v>0.46</v>
       </c>
       <c r="G139" t="n">
-        <v>0.16</v>
+        <v>0.47</v>
       </c>
       <c r="H139" t="n">
         <v>0.93</v>
@@ -9201,7 +9201,7 @@
         <v>0.65</v>
       </c>
       <c r="J139" t="n">
-        <v>0.3575</v>
+        <v>0.586</v>
       </c>
       <c r="K139" t="n">
         <v>3</v>
@@ -9252,10 +9252,10 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>0.41</v>
+        <v>0.76</v>
       </c>
       <c r="G140" t="n">
-        <v>0.42</v>
+        <v>0.76</v>
       </c>
       <c r="H140" t="n">
         <v>0.61</v>
@@ -9264,10 +9264,10 @@
         <v>0.65</v>
       </c>
       <c r="J140" t="n">
-        <v>0.4895</v>
+        <v>0.7135</v>
       </c>
       <c r="K140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L140" t="n">
         <v>2100</v>
@@ -9315,10 +9315,10 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>0.29</v>
+        <v>0.68</v>
       </c>
       <c r="G141" t="n">
-        <v>0.33</v>
+        <v>0.68</v>
       </c>
       <c r="H141" t="n">
         <v>0.93</v>
@@ -9327,10 +9327,10 @@
         <v>0.65</v>
       </c>
       <c r="J141" t="n">
-        <v>0.486</v>
+        <v>0.7255</v>
       </c>
       <c r="K141" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L141" t="n">
         <v>2100</v>
@@ -9378,10 +9378,10 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>0.19</v>
+        <v>0.61</v>
       </c>
       <c r="G142" t="n">
-        <v>0.27</v>
+        <v>0.62</v>
       </c>
       <c r="H142" t="n">
         <v>0.86</v>
@@ -9390,7 +9390,7 @@
         <v>0.65</v>
       </c>
       <c r="J142" t="n">
-        <v>0.421</v>
+        <v>0.6695</v>
       </c>
       <c r="K142" t="n">
         <v>3</v>
@@ -9441,10 +9441,10 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>0.2</v>
+        <v>0.63</v>
       </c>
       <c r="G143" t="n">
-        <v>0.22</v>
+        <v>0.64</v>
       </c>
       <c r="H143" t="n">
         <v>0.7</v>
@@ -9453,7 +9453,7 @@
         <v>0.65</v>
       </c>
       <c r="J143" t="n">
-        <v>0.3745</v>
+        <v>0.6505</v>
       </c>
       <c r="K143" t="n">
         <v>1</v>
@@ -9504,10 +9504,10 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>0.1</v>
+        <v>0.55</v>
       </c>
       <c r="G144" t="n">
-        <v>0.14</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H144" t="n">
         <v>0.93</v>
@@ -9516,7 +9516,7 @@
         <v>0.65</v>
       </c>
       <c r="J144" t="n">
-        <v>0.3625</v>
+        <v>0.6445</v>
       </c>
       <c r="K144" t="n">
         <v>2</v>
@@ -9567,10 +9567,10 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="G145" t="n">
-        <v>0</v>
+        <v>0.44</v>
       </c>
       <c r="H145" t="n">
         <v>0.7</v>
@@ -9579,7 +9579,7 @@
         <v>0.65</v>
       </c>
       <c r="J145" t="n">
-        <v>0.2375</v>
+        <v>0.5175</v>
       </c>
       <c r="K145" t="n">
         <v>3</v>
@@ -9630,10 +9630,10 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="G146" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="H146" t="n">
         <v>0.61</v>
@@ -9642,7 +9642,7 @@
         <v>0.65</v>
       </c>
       <c r="J146" t="n">
-        <v>0.5835</v>
+        <v>0.785</v>
       </c>
       <c r="K146" t="n">
         <v>2</v>
@@ -9693,10 +9693,10 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>0.49</v>
+        <v>0.8</v>
       </c>
       <c r="G147" t="n">
-        <v>0.49</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H147" t="n">
         <v>0.86</v>
@@ -9705,7 +9705,7 @@
         <v>0.65</v>
       </c>
       <c r="J147" t="n">
-        <v>0.588</v>
+        <v>0.793</v>
       </c>
       <c r="K147" t="n">
         <v>1</v>
@@ -9756,10 +9756,10 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>0.39</v>
+        <v>0.72</v>
       </c>
       <c r="G148" t="n">
-        <v>0.4</v>
+        <v>0.72</v>
       </c>
       <c r="H148" t="n">
         <v>0.86</v>
@@ -9768,7 +9768,7 @@
         <v>0.65</v>
       </c>
       <c r="J148" t="n">
-        <v>0.5265</v>
+        <v>0.7375</v>
       </c>
       <c r="K148" t="n">
         <v>3</v>
@@ -9819,10 +9819,10 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>0.31</v>
+        <v>0.26</v>
       </c>
       <c r="G149" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="H149" t="n">
         <v>0.45</v>
@@ -9831,7 +9831,7 @@
         <v>0.71</v>
       </c>
       <c r="J149" t="n">
-        <v>0.4015</v>
+        <v>0.369</v>
       </c>
       <c r="K149" t="n">
         <v>3</v>
@@ -9882,10 +9882,10 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="G150" t="n">
-        <v>0.41</v>
+        <v>0.34</v>
       </c>
       <c r="H150" t="n">
         <v>0.93</v>
@@ -9894,7 +9894,7 @@
         <v>0.84</v>
       </c>
       <c r="J150" t="n">
-        <v>0.5755</v>
+        <v>0.53</v>
       </c>
       <c r="K150" t="n">
         <v>2</v>
@@ -9945,10 +9945,10 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="G151" t="n">
-        <v>0.49</v>
+        <v>0.42</v>
       </c>
       <c r="H151" t="n">
         <v>0.67</v>
@@ -9957,7 +9957,7 @@
         <v>0.84</v>
       </c>
       <c r="J151" t="n">
-        <v>0.5755</v>
+        <v>0.53</v>
       </c>
       <c r="K151" t="n">
         <v>1</v>
@@ -10008,10 +10008,10 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="G152" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="H152" t="n">
         <v>0.86</v>
@@ -10020,7 +10020,7 @@
         <v>0.84</v>
       </c>
       <c r="J152" t="n">
-        <v>0.5745</v>
+        <v>0.5355</v>
       </c>
       <c r="K152" t="n">
         <v>3</v>
@@ -10071,10 +10071,10 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>0.49</v>
+        <v>0.42</v>
       </c>
       <c r="G153" t="n">
-        <v>0.5</v>
+        <v>0.43</v>
       </c>
       <c r="H153" t="n">
         <v>0.86</v>
@@ -10083,7 +10083,7 @@
         <v>0.84</v>
       </c>
       <c r="J153" t="n">
-        <v>0.62</v>
+        <v>0.5745</v>
       </c>
       <c r="K153" t="n">
         <v>1</v>
@@ -10134,10 +10134,10 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="G154" t="n">
-        <v>0.57</v>
+        <v>0.49</v>
       </c>
       <c r="H154" t="n">
         <v>0.51</v>
@@ -10146,7 +10146,7 @@
         <v>0.87</v>
       </c>
       <c r="J154" t="n">
-        <v>0.6</v>
+        <v>0.548</v>
       </c>
       <c r="K154" t="n">
         <v>2</v>
@@ -10197,10 +10197,10 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
       <c r="G155" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
       <c r="H155" t="n">
         <v>0.29</v>
@@ -10209,7 +10209,7 @@
         <v>0.65</v>
       </c>
       <c r="J155" t="n">
-        <v>0.6885</v>
+        <v>0.617</v>
       </c>
       <c r="K155" t="n">
         <v>3</v>
@@ -10260,10 +10260,10 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="G156" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H156" t="n">
         <v>0.51</v>
@@ -10272,7 +10272,7 @@
         <v>0.8</v>
       </c>
       <c r="J156" t="n">
-        <v>0.768</v>
+        <v>0.6965</v>
       </c>
       <c r="K156" t="n">
         <v>2</v>
@@ -10323,10 +10323,10 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>0.86</v>
+        <v>0.75</v>
       </c>
       <c r="G157" t="n">
-        <v>0.86</v>
+        <v>0.75</v>
       </c>
       <c r="H157" t="n">
         <v>0.7</v>
@@ -10335,7 +10335,7 @@
         <v>0.87</v>
       </c>
       <c r="J157" t="n">
-        <v>0.8295</v>
+        <v>0.758</v>
       </c>
       <c r="K157" t="n">
         <v>1</v>
@@ -10386,10 +10386,10 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>0.84</v>
+        <v>0.92</v>
       </c>
       <c r="G158" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="H158" t="n">
         <v>0.61</v>
@@ -10398,7 +10398,7 @@
         <v>0.65</v>
       </c>
       <c r="J158" t="n">
-        <v>0.762</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="K158" t="n">
         <v>3</v>
@@ -10449,10 +10449,10 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="G159" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="H159" t="n">
         <v>0.86</v>
@@ -10461,10 +10461,10 @@
         <v>0.65</v>
       </c>
       <c r="J159" t="n">
-        <v>0.796</v>
+        <v>0.848</v>
       </c>
       <c r="K159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L159" t="n">
         <v>980</v>
@@ -10512,10 +10512,10 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>0.78</v>
+        <v>0.87</v>
       </c>
       <c r="G160" t="n">
-        <v>0.78</v>
+        <v>0.87</v>
       </c>
       <c r="H160" t="n">
         <v>0.93</v>
@@ -10524,10 +10524,10 @@
         <v>0.65</v>
       </c>
       <c r="J160" t="n">
-        <v>0.7905</v>
+        <v>0.849</v>
       </c>
       <c r="K160" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L160" t="n">
         <v>980</v>
@@ -10641,7 +10641,7 @@
         <v>1</v>
       </c>
       <c r="G162" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="H162" t="n">
         <v>0.76</v>
@@ -10650,7 +10650,7 @@
         <v>0.77</v>
       </c>
       <c r="J162" t="n">
-        <v>0.914</v>
+        <v>0.9175</v>
       </c>
       <c r="K162" t="n">
         <v>2</v>
@@ -10701,10 +10701,10 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="G163" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="H163" t="n">
         <v>1</v>
@@ -10713,7 +10713,7 @@
         <v>0.77</v>
       </c>
       <c r="J163" t="n">
-        <v>0.9295</v>
+        <v>0.9655</v>
       </c>
       <c r="K163" t="n">
         <v>1</v>
@@ -10764,10 +10764,10 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="G164" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="H164" t="n">
         <v>0</v>
@@ -10776,7 +10776,7 @@
         <v>0.48</v>
       </c>
       <c r="J164" t="n">
-        <v>0.5595</v>
+        <v>0.4945</v>
       </c>
       <c r="K164" t="n">
         <v>3</v>
@@ -10827,10 +10827,10 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="G165" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="H165" t="n">
         <v>0.7</v>
@@ -10839,7 +10839,7 @@
         <v>0.87</v>
       </c>
       <c r="J165" t="n">
-        <v>0.8165</v>
+        <v>0.745</v>
       </c>
       <c r="K165" t="n">
         <v>2</v>
@@ -10890,10 +10890,10 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G166" t="n">
-        <v>0.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H166" t="n">
         <v>0.86</v>
@@ -10902,7 +10902,7 @@
         <v>0.84</v>
       </c>
       <c r="J166" t="n">
-        <v>0.9055</v>
+        <v>0.8245</v>
       </c>
       <c r="K166" t="n">
         <v>1</v>
@@ -10953,10 +10953,10 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="G167" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="H167" t="n">
         <v>0.7</v>
@@ -10965,7 +10965,7 @@
         <v>0.87</v>
       </c>
       <c r="J167" t="n">
-        <v>0.862</v>
+        <v>0.784</v>
       </c>
       <c r="K167" t="n">
         <v>3</v>
@@ -11016,10 +11016,10 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G168" t="n">
-        <v>0.93</v>
+        <v>0.82</v>
       </c>
       <c r="H168" t="n">
         <v>1</v>
@@ -11028,7 +11028,7 @@
         <v>0.87</v>
       </c>
       <c r="J168" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.8605</v>
       </c>
       <c r="K168" t="n">
         <v>1</v>
@@ -11079,10 +11079,10 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>0.96</v>
+        <v>0.83</v>
       </c>
       <c r="G169" t="n">
-        <v>0.95</v>
+        <v>0.83</v>
       </c>
       <c r="H169" t="n">
         <v>0.78</v>
@@ -11091,7 +11091,7 @@
         <v>0.87</v>
       </c>
       <c r="J169" t="n">
-        <v>0.907</v>
+        <v>0.826</v>
       </c>
       <c r="K169" t="n">
         <v>2</v>
@@ -11142,10 +11142,10 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="G170" t="n">
-        <v>0.48</v>
+        <v>0.41</v>
       </c>
       <c r="H170" t="n">
         <v>0.67</v>
@@ -11154,7 +11154,7 @@
         <v>0.77</v>
       </c>
       <c r="J170" t="n">
-        <v>0.5585</v>
+        <v>0.513</v>
       </c>
       <c r="K170" t="n">
         <v>3</v>
@@ -11205,10 +11205,10 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>0.52</v>
+        <v>0.44</v>
       </c>
       <c r="G171" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="H171" t="n">
         <v>1</v>
@@ -11217,7 +11217,7 @@
         <v>0.77</v>
       </c>
       <c r="J171" t="n">
-        <v>0.657</v>
+        <v>0.6085</v>
       </c>
       <c r="K171" t="n">
         <v>1</v>
@@ -11268,10 +11268,10 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>0.58</v>
+        <v>0.49</v>
       </c>
       <c r="G172" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="H172" t="n">
         <v>0.67</v>
@@ -11280,7 +11280,7 @@
         <v>0.84</v>
       </c>
       <c r="J172" t="n">
-        <v>0.637</v>
+        <v>0.582</v>
       </c>
       <c r="K172" t="n">
         <v>2</v>
@@ -11331,10 +11331,10 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="G173" t="n">
-        <v>0.64</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H173" t="n">
         <v>0.73</v>
@@ -11343,7 +11343,7 @@
         <v>0.84</v>
       </c>
       <c r="J173" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.633</v>
       </c>
       <c r="K173" t="n">
         <v>3</v>
@@ -11394,10 +11394,10 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="G174" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="H174" t="n">
         <v>0.92</v>
@@ -11406,7 +11406,7 @@
         <v>0.84</v>
       </c>
       <c r="J174" t="n">
-        <v>0.7585</v>
+        <v>0.697</v>
       </c>
       <c r="K174" t="n">
         <v>1</v>
@@ -11457,10 +11457,10 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="G175" t="n">
-        <v>0.73</v>
+        <v>0.63</v>
       </c>
       <c r="H175" t="n">
         <v>0.51</v>
@@ -11469,7 +11469,7 @@
         <v>0.87</v>
       </c>
       <c r="J175" t="n">
-        <v>0.707</v>
+        <v>0.642</v>
       </c>
       <c r="K175" t="n">
         <v>2</v>
@@ -11520,10 +11520,10 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>0.73</v>
+        <v>0.98</v>
       </c>
       <c r="G176" t="n">
-        <v>0.73</v>
+        <v>0.98</v>
       </c>
       <c r="H176" t="n">
         <v>0.15</v>
@@ -11532,7 +11532,7 @@
         <v>0.65</v>
       </c>
       <c r="J176" t="n">
-        <v>0.602</v>
+        <v>0.7645</v>
       </c>
       <c r="K176" t="n">
         <v>3</v>
@@ -11583,10 +11583,10 @@
         </is>
       </c>
       <c r="F177" t="n">
-        <v>0.65</v>
+        <v>0.9</v>
       </c>
       <c r="G177" t="n">
-        <v>0.65</v>
+        <v>0.9</v>
       </c>
       <c r="H177" t="n">
         <v>0.61</v>
@@ -11595,7 +11595,7 @@
         <v>0.65</v>
       </c>
       <c r="J177" t="n">
-        <v>0.642</v>
+        <v>0.8045</v>
       </c>
       <c r="K177" t="n">
         <v>2</v>
@@ -11646,10 +11646,10 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>0.58</v>
+        <v>0.85</v>
       </c>
       <c r="G178" t="n">
-        <v>0.59</v>
+        <v>0.85</v>
       </c>
       <c r="H178" t="n">
         <v>0.86</v>
@@ -11658,7 +11658,7 @@
         <v>0.65</v>
       </c>
       <c r="J178" t="n">
-        <v>0.65</v>
+        <v>0.822</v>
       </c>
       <c r="K178" t="n">
         <v>1</v>
@@ -11898,10 +11898,10 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>0.57</v>
+        <v>0.86</v>
       </c>
       <c r="G182" t="n">
-        <v>0.58</v>
+        <v>0.86</v>
       </c>
       <c r="H182" t="n">
         <v>0.41</v>
@@ -11910,7 +11910,7 @@
         <v>0.65</v>
       </c>
       <c r="J182" t="n">
-        <v>0.5535</v>
+        <v>0.7385</v>
       </c>
       <c r="K182" t="n">
         <v>3</v>
@@ -11961,10 +11961,10 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>0.51</v>
+        <v>0.8</v>
       </c>
       <c r="G183" t="n">
-        <v>0.51</v>
+        <v>0.8</v>
       </c>
       <c r="H183" t="n">
         <v>0.7</v>
@@ -11973,7 +11973,7 @@
         <v>0.65</v>
       </c>
       <c r="J183" t="n">
-        <v>0.569</v>
+        <v>0.7575</v>
       </c>
       <c r="K183" t="n">
         <v>2</v>
@@ -12024,10 +12024,10 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>0.44</v>
+        <v>0.74</v>
       </c>
       <c r="G184" t="n">
-        <v>0.45</v>
+        <v>0.74</v>
       </c>
       <c r="H184" t="n">
         <v>0.93</v>
@@ -12036,7 +12036,7 @@
         <v>0.65</v>
       </c>
       <c r="J184" t="n">
-        <v>0.573</v>
+        <v>0.7645</v>
       </c>
       <c r="K184" t="n">
         <v>1</v>
@@ -12087,10 +12087,10 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>0.38</v>
+        <v>0.73</v>
       </c>
       <c r="G185" t="n">
-        <v>0.4</v>
+        <v>0.74</v>
       </c>
       <c r="H185" t="n">
         <v>0.02</v>
@@ -12099,7 +12099,7 @@
         <v>0.55</v>
       </c>
       <c r="J185" t="n">
-        <v>0.3405</v>
+        <v>0.5645</v>
       </c>
       <c r="K185" t="n">
         <v>3</v>
@@ -12150,10 +12150,10 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>0.31</v>
+        <v>0.67</v>
       </c>
       <c r="G186" t="n">
-        <v>0.32</v>
+        <v>0.67</v>
       </c>
       <c r="H186" t="n">
         <v>0.45</v>
@@ -12162,7 +12162,7 @@
         <v>0.65</v>
       </c>
       <c r="J186" t="n">
-        <v>0.3925</v>
+        <v>0.623</v>
       </c>
       <c r="K186" t="n">
         <v>2</v>
@@ -12213,10 +12213,10 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>0.22</v>
+        <v>0.6</v>
       </c>
       <c r="G187" t="n">
-        <v>0.25</v>
+        <v>0.61</v>
       </c>
       <c r="H187" t="n">
         <v>0.76</v>
@@ -12225,7 +12225,7 @@
         <v>0.65</v>
       </c>
       <c r="J187" t="n">
-        <v>0.403</v>
+        <v>0.643</v>
       </c>
       <c r="K187" t="n">
         <v>1</v>
@@ -12276,10 +12276,10 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="G188" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="H188" t="n">
         <v>0</v>
@@ -12288,7 +12288,7 @@
         <v>0.15</v>
       </c>
       <c r="J188" t="n">
-        <v>0.5685</v>
+        <v>0.666</v>
       </c>
       <c r="K188" t="n">
         <v>3</v>
@@ -12339,10 +12339,10 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>0.8</v>
+        <v>0.96</v>
       </c>
       <c r="G189" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="H189" t="n">
         <v>0</v>
@@ -12351,7 +12351,7 @@
         <v>0.44</v>
       </c>
       <c r="J189" t="n">
-        <v>0.586</v>
+        <v>0.6865</v>
       </c>
       <c r="K189" t="n">
         <v>2</v>
@@ -12402,10 +12402,10 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>0.76</v>
+        <v>0.92</v>
       </c>
       <c r="G190" t="n">
-        <v>0.76</v>
+        <v>0.92</v>
       </c>
       <c r="H190" t="n">
         <v>0.41</v>
@@ -12414,7 +12414,7 @@
         <v>0.65</v>
       </c>
       <c r="J190" t="n">
-        <v>0.6735</v>
+        <v>0.7775</v>
       </c>
       <c r="K190" t="n">
         <v>1</v>
@@ -12465,10 +12465,10 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>0.82</v>
+        <v>1</v>
       </c>
       <c r="G191" t="n">
-        <v>0.82</v>
+        <v>1</v>
       </c>
       <c r="H191" t="n">
         <v>0.41</v>
@@ -12477,7 +12477,7 @@
         <v>0.65</v>
       </c>
       <c r="J191" t="n">
-        <v>0.7125</v>
+        <v>0.8295</v>
       </c>
       <c r="K191" t="n">
         <v>3</v>
@@ -12528,10 +12528,10 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>0.77</v>
+        <v>0.96</v>
       </c>
       <c r="G192" t="n">
-        <v>0.77</v>
+        <v>0.96</v>
       </c>
       <c r="H192" t="n">
         <v>0.7</v>
@@ -12540,7 +12540,7 @@
         <v>0.65</v>
       </c>
       <c r="J192" t="n">
-        <v>0.738</v>
+        <v>0.8615</v>
       </c>
       <c r="K192" t="n">
         <v>2</v>
@@ -12591,10 +12591,10 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="G193" t="n">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="H193" t="n">
         <v>0.93</v>
@@ -12603,7 +12603,7 @@
         <v>0.65</v>
       </c>
       <c r="J193" t="n">
-        <v>0.7514999999999999</v>
+        <v>0.8815</v>
       </c>
       <c r="K193" t="n">
         <v>1</v>
@@ -12654,10 +12654,10 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>0.25</v>
+        <v>0.61</v>
       </c>
       <c r="G194" t="n">
-        <v>0.28</v>
+        <v>0.62</v>
       </c>
       <c r="H194" t="n">
         <v>0</v>
@@ -12666,7 +12666,7 @@
         <v>0.31</v>
       </c>
       <c r="J194" t="n">
-        <v>0.2195</v>
+        <v>0.4465</v>
       </c>
       <c r="K194" t="n">
         <v>3</v>
@@ -12717,10 +12717,10 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>0.15</v>
+        <v>0.55</v>
       </c>
       <c r="G195" t="n">
-        <v>0.21</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H195" t="n">
         <v>0.29</v>
@@ -12729,7 +12729,7 @@
         <v>0.65</v>
       </c>
       <c r="J195" t="n">
-        <v>0.274</v>
+        <v>0.5165</v>
       </c>
       <c r="K195" t="n">
         <v>2</v>
@@ -12780,10 +12780,10 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="G196" t="n">
-        <v>0.14</v>
+        <v>0.49</v>
       </c>
       <c r="H196" t="n">
         <v>0.61</v>
@@ -12792,7 +12792,7 @@
         <v>0.65</v>
       </c>
       <c r="J196" t="n">
-        <v>0.2895</v>
+        <v>0.535</v>
       </c>
       <c r="K196" t="n">
         <v>1</v>
@@ -12843,10 +12843,10 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>0.17</v>
+        <v>0.57</v>
       </c>
       <c r="G197" t="n">
-        <v>0.3</v>
+        <v>0.57</v>
       </c>
       <c r="H197" t="n">
         <v>0.15</v>
@@ -12855,7 +12855,7 @@
         <v>0.55</v>
       </c>
       <c r="J197" t="n">
-        <v>0.2685</v>
+        <v>0.483</v>
       </c>
       <c r="K197" t="n">
         <v>3</v>
@@ -12906,10 +12906,10 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>0.1</v>
+        <v>0.51</v>
       </c>
       <c r="G198" t="n">
-        <v>0.24</v>
+        <v>0.52</v>
       </c>
       <c r="H198" t="n">
         <v>0.51</v>
@@ -12918,7 +12918,7 @@
         <v>0.65</v>
       </c>
       <c r="J198" t="n">
-        <v>0.3135</v>
+        <v>0.5345</v>
       </c>
       <c r="K198" t="n">
         <v>2</v>
@@ -12969,10 +12969,10 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>0.06</v>
+        <v>0.46</v>
       </c>
       <c r="G199" t="n">
-        <v>0.18</v>
+        <v>0.47</v>
       </c>
       <c r="H199" t="n">
         <v>0.78</v>
@@ -12981,7 +12981,7 @@
         <v>0.65</v>
       </c>
       <c r="J199" t="n">
-        <v>0.3345</v>
+        <v>0.556</v>
       </c>
       <c r="K199" t="n">
         <v>1</v>
@@ -13032,10 +13032,10 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>0.76</v>
+        <v>0.96</v>
       </c>
       <c r="G200" t="n">
-        <v>0.75</v>
+        <v>0.96</v>
       </c>
       <c r="H200" t="n">
         <v>0</v>
@@ -13044,7 +13044,7 @@
         <v>0.31</v>
       </c>
       <c r="J200" t="n">
-        <v>0.537</v>
+        <v>0.6705</v>
       </c>
       <c r="K200" t="n">
         <v>3</v>
@@ -13095,10 +13095,10 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>0.7</v>
+        <v>0.92</v>
       </c>
       <c r="G201" t="n">
-        <v>0.7</v>
+        <v>0.92</v>
       </c>
       <c r="H201" t="n">
         <v>0.29</v>
@@ -13107,7 +13107,7 @@
         <v>0.65</v>
       </c>
       <c r="J201" t="n">
-        <v>0.6105</v>
+        <v>0.7534999999999999</v>
       </c>
       <c r="K201" t="n">
         <v>2</v>
@@ -13158,10 +13158,10 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>0.65</v>
+        <v>0.87</v>
       </c>
       <c r="G202" t="n">
-        <v>0.65</v>
+        <v>0.87</v>
       </c>
       <c r="H202" t="n">
         <v>0.61</v>
@@ -13170,7 +13170,7 @@
         <v>0.65</v>
       </c>
       <c r="J202" t="n">
-        <v>0.642</v>
+        <v>0.785</v>
       </c>
       <c r="K202" t="n">
         <v>1</v>
@@ -13221,10 +13221,10 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>0.09</v>
+        <v>0.53</v>
       </c>
       <c r="G203" t="n">
-        <v>0.11</v>
+        <v>0.54</v>
       </c>
       <c r="H203" t="n">
         <v>0</v>
@@ -13233,7 +13233,7 @@
         <v>0.55</v>
       </c>
       <c r="J203" t="n">
-        <v>0.148</v>
+        <v>0.4305</v>
       </c>
       <c r="K203" t="n">
         <v>3</v>
@@ -13284,10 +13284,10 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="G204" t="n">
-        <v>0.03</v>
+        <v>0.46</v>
       </c>
       <c r="H204" t="n">
         <v>0.38</v>
@@ -13296,7 +13296,7 @@
         <v>0.65</v>
       </c>
       <c r="J204" t="n">
-        <v>0.184</v>
+        <v>0.4695</v>
       </c>
       <c r="K204" t="n">
         <v>2</v>
@@ -13347,10 +13347,10 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
       <c r="G205" t="n">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="H205" t="n">
         <v>0.73</v>
@@ -13359,7 +13359,7 @@
         <v>0.65</v>
       </c>
       <c r="J205" t="n">
-        <v>0.2435</v>
+        <v>0.494</v>
       </c>
       <c r="K205" t="n">
         <v>1</v>
@@ -13410,10 +13410,10 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>0.55</v>
+        <v>0.47</v>
       </c>
       <c r="G206" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="H206" t="n">
         <v>0.78</v>
@@ -13422,7 +13422,7 @@
         <v>0.84</v>
       </c>
       <c r="J206" t="n">
-        <v>0.643</v>
+        <v>0.591</v>
       </c>
       <c r="K206" t="n">
         <v>3</v>
@@ -13473,10 +13473,10 @@
         </is>
       </c>
       <c r="F207" t="n">
-        <v>0.6</v>
+        <v>0.51</v>
       </c>
       <c r="G207" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="H207" t="n">
         <v>1</v>
@@ -13485,7 +13485,7 @@
         <v>0.84</v>
       </c>
       <c r="J207" t="n">
-        <v>0.716</v>
+        <v>0.661</v>
       </c>
       <c r="K207" t="n">
         <v>1</v>
@@ -13536,10 +13536,10 @@
         </is>
       </c>
       <c r="F208" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="G208" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H208" t="n">
         <v>0.78</v>
@@ -13548,7 +13548,7 @@
         <v>0.84</v>
       </c>
       <c r="J208" t="n">
-        <v>0.7015</v>
+        <v>0.643</v>
       </c>
       <c r="K208" t="n">
         <v>2</v>
@@ -13599,10 +13599,10 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>0.65</v>
+        <v>0.55</v>
       </c>
       <c r="G209" t="n">
-        <v>0.65</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H209" t="n">
         <v>0.86</v>
@@ -13611,7 +13611,7 @@
         <v>0.84</v>
       </c>
       <c r="J209" t="n">
-        <v>0.7205</v>
+        <v>0.659</v>
       </c>
       <c r="K209" t="n">
         <v>1</v>
@@ -13662,10 +13662,10 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="G210" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="H210" t="n">
         <v>0.61</v>
@@ -13674,7 +13674,7 @@
         <v>0.84</v>
       </c>
       <c r="J210" t="n">
-        <v>0.6965</v>
+        <v>0.635</v>
       </c>
       <c r="K210" t="n">
         <v>2</v>
@@ -13725,10 +13725,10 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>0.72</v>
+        <v>0.62</v>
       </c>
       <c r="G211" t="n">
-        <v>0.72</v>
+        <v>0.63</v>
       </c>
       <c r="H211" t="n">
         <v>0.29</v>
@@ -13737,7 +13737,7 @@
         <v>0.65</v>
       </c>
       <c r="J211" t="n">
-        <v>0.6235000000000001</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="K211" t="n">
         <v>3</v>

</xml_diff>